<commit_message>
Agregada funcion de no incluir en depreciacion
</commit_message>
<xml_diff>
--- a/ControlActivosTI/templates/actas/5. F-TI-05 - Acta de Recepción de Equipos y Servicios de Tecnología.xlsx
+++ b/ControlActivosTI/templates/actas/5. F-TI-05 - Acta de Recepción de Equipos y Servicios de Tecnología.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto\ControlActivosTI\ControlActivosTI\templates\actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED599BC-BFF8-456D-A7C4-5A583CECA9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3E078C-632B-4CB3-8496-6DA00CD40281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14290" yWindow="-1820" windowWidth="19420" windowHeight="10300" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
+    <workbookView xWindow="14290" yWindow="-1820" windowWidth="19420" windowHeight="11020" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1115,50 +1115,143 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1168,6 +1261,105 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1190,15 +1382,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1206,9 +1389,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1217,230 +1397,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1875,42 +1875,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="90" t="e" vm="1">
+      <c r="B1" s="33" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C1" s="91"/>
-      <c r="D1" s="94" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="97" t="s">
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="99" t="s">
+      <c r="I1" s="44" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="92"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="101" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="102"/>
-      <c r="F2" s="102"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="100"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="45"/>
     </row>
     <row r="3" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="92"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
-      <c r="G3" s="106"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="51"/>
       <c r="H3" s="16" t="s">
         <v>2</v>
       </c>
@@ -1919,120 +1919,120 @@
       </c>
     </row>
     <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="92"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="106"/>
-      <c r="H4" s="110" t="s">
+      <c r="B4" s="35"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="51"/>
+      <c r="H4" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="112">
+      <c r="I4" s="57">
         <v>46097</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="93"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="109"/>
-      <c r="H5" s="111"/>
-      <c r="I5" s="113"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="58"/>
     </row>
     <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="81" t="s">
+      <c r="B6" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="82"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="125"/>
-      <c r="F6" s="126"/>
-      <c r="G6" s="126"/>
-      <c r="H6" s="126"/>
-      <c r="I6" s="127"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="78"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="124" t="s">
+      <c r="B7" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="86"/>
-      <c r="D7" s="86"/>
-      <c r="E7" s="86"/>
-      <c r="F7" s="86"/>
-      <c r="G7" s="86"/>
-      <c r="H7" s="86"/>
-      <c r="I7" s="87"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="69"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="69"/>
+      <c r="I7" s="70"/>
     </row>
     <row r="8" spans="2:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="44"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="46"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="73"/>
     </row>
     <row r="9" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="44"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="46"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="72"/>
+      <c r="H9" s="72"/>
+      <c r="I9" s="73"/>
     </row>
     <row r="10" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="123" t="s">
+      <c r="B10" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="119"/>
-      <c r="D10" s="119"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="119" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="53"/>
+      <c r="I10" s="20"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="114" t="s">
+      <c r="B11" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="115"/>
-      <c r="D11" s="115"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="117"/>
-      <c r="G11" s="118"/>
-      <c r="H11" s="119"/>
-      <c r="I11" s="53"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="20"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="120" t="s">
+      <c r="B12" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="121"/>
-      <c r="D12" s="121"/>
-      <c r="E12" s="121"/>
-      <c r="F12" s="121"/>
-      <c r="G12" s="121"/>
-      <c r="H12" s="121"/>
-      <c r="I12" s="122"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="88" t="s">
+      <c r="B13" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="89"/>
-      <c r="D13" s="89" t="s">
+      <c r="C13" s="75"/>
+      <c r="D13" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="89"/>
+      <c r="E13" s="75"/>
       <c r="F13" s="3" t="s">
         <v>15</v>
       </c>
@@ -2047,83 +2047,83 @@
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="85"/>
-      <c r="C14" s="84"/>
-      <c r="D14" s="84"/>
-      <c r="E14" s="84"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="85"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="84"/>
-      <c r="E15" s="84"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="4"/>
     </row>
     <row r="16" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="85"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="84"/>
-      <c r="E16" s="84"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="85"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="85"/>
-      <c r="C18" s="84"/>
-      <c r="D18" s="84"/>
-      <c r="E18" s="84"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="4"/>
     </row>
     <row r="19" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="85"/>
-      <c r="C19" s="84"/>
-      <c r="D19" s="84"/>
-      <c r="E19" s="84"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="4"/>
     </row>
     <row r="20" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="36"/>
+      <c r="C20" s="66"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="66"/>
+      <c r="G20" s="66"/>
+      <c r="H20" s="66"/>
+      <c r="I20" s="67"/>
     </row>
     <row r="21" spans="2:9" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
+      <c r="C21" s="104"/>
+      <c r="D21" s="104"/>
       <c r="E21" s="5" t="s">
         <v>31</v>
       </c>
@@ -2133,17 +2133,17 @@
       <c r="G21" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="H21" s="37" t="s">
+      <c r="H21" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="38"/>
+      <c r="I21" s="102"/>
     </row>
     <row r="22" spans="2:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="47" t="s">
+      <c r="B22" s="108" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
+      <c r="C22" s="109"/>
+      <c r="D22" s="109"/>
       <c r="E22" s="12" t="b">
         <v>0</v>
       </c>
@@ -2153,15 +2153,15 @@
       <c r="G22" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="H22" s="51"/>
-      <c r="I22" s="52"/>
+      <c r="H22" s="111"/>
+      <c r="I22" s="112"/>
     </row>
     <row r="23" spans="2:9" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="49" t="s">
+      <c r="B23" s="110" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="50"/>
-      <c r="D23" s="50"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
       <c r="E23" s="6" t="b">
         <v>0</v>
       </c>
@@ -2171,15 +2171,15 @@
       <c r="G23" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H23" s="50"/>
-      <c r="I23" s="53"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="20"/>
     </row>
     <row r="24" spans="2:9" s="8" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="113" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
+      <c r="C24" s="114"/>
+      <c r="D24" s="115"/>
       <c r="E24" s="6" t="b">
         <v>0</v>
       </c>
@@ -2189,15 +2189,15 @@
       <c r="G24" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="22"/>
-      <c r="I24" s="23"/>
+      <c r="H24" s="116"/>
+      <c r="I24" s="117"/>
     </row>
     <row r="25" spans="2:9" s="8" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="113" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="21"/>
+      <c r="C25" s="114"/>
+      <c r="D25" s="115"/>
       <c r="E25" s="6" t="b">
         <v>0</v>
       </c>
@@ -2207,15 +2207,15 @@
       <c r="G25" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23"/>
+      <c r="H25" s="116"/>
+      <c r="I25" s="117"/>
     </row>
     <row r="26" spans="2:9" s="8" customFormat="1" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="118" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26"/>
+      <c r="C26" s="119"/>
+      <c r="D26" s="120"/>
       <c r="E26" s="14" t="b">
         <v>0</v>
       </c>
@@ -2225,15 +2225,15 @@
       <c r="G26" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="H26" s="27"/>
-      <c r="I26" s="28"/>
+      <c r="H26" s="121"/>
+      <c r="I26" s="122"/>
     </row>
     <row r="27" spans="2:9" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="123" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="31"/>
+      <c r="C27" s="124"/>
+      <c r="D27" s="125"/>
       <c r="E27" s="10" t="b">
         <v>0</v>
       </c>
@@ -2243,15 +2243,15 @@
       <c r="G27" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H27" s="32"/>
-      <c r="I27" s="33"/>
+      <c r="H27" s="126"/>
+      <c r="I27" s="127"/>
     </row>
     <row r="28" spans="2:9" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="113" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="21"/>
+      <c r="C28" s="114"/>
+      <c r="D28" s="115"/>
       <c r="E28" s="6" t="b">
         <v>0</v>
       </c>
@@ -2261,15 +2261,15 @@
       <c r="G28" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H28" s="22"/>
-      <c r="I28" s="23"/>
+      <c r="H28" s="116"/>
+      <c r="I28" s="117"/>
     </row>
     <row r="29" spans="2:9" s="8" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="113" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="21"/>
+      <c r="C29" s="114"/>
+      <c r="D29" s="115"/>
       <c r="E29" s="6" t="b">
         <v>0</v>
       </c>
@@ -2279,384 +2279,409 @@
       <c r="G29" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="H29" s="22"/>
-      <c r="I29" s="23"/>
+      <c r="H29" s="116"/>
+      <c r="I29" s="117"/>
     </row>
     <row r="30" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B30" s="34" t="s">
+      <c r="B30" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35"/>
-      <c r="H30" s="35"/>
-      <c r="I30" s="36"/>
+      <c r="C30" s="66"/>
+      <c r="D30" s="66"/>
+      <c r="E30" s="66"/>
+      <c r="F30" s="66"/>
+      <c r="G30" s="66"/>
+      <c r="H30" s="66"/>
+      <c r="I30" s="67"/>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B31" s="44" t="s">
+      <c r="B31" s="71" t="s">
         <v>24</v>
       </c>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="46"/>
+      <c r="C31" s="72"/>
+      <c r="D31" s="72"/>
+      <c r="E31" s="72"/>
+      <c r="F31" s="72"/>
+      <c r="G31" s="72"/>
+      <c r="H31" s="72"/>
+      <c r="I31" s="73"/>
     </row>
     <row r="32" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="44"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="46"/>
+      <c r="B32" s="71"/>
+      <c r="C32" s="72"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="72"/>
+      <c r="G32" s="72"/>
+      <c r="H32" s="72"/>
+      <c r="I32" s="73"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
-      <c r="I33" s="46"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="72"/>
+      <c r="F33" s="72"/>
+      <c r="G33" s="72"/>
+      <c r="H33" s="72"/>
+      <c r="I33" s="73"/>
     </row>
     <row r="34" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="44"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="45"/>
-      <c r="I34" s="46"/>
+      <c r="B34" s="71"/>
+      <c r="C34" s="72"/>
+      <c r="D34" s="72"/>
+      <c r="E34" s="72"/>
+      <c r="F34" s="72"/>
+      <c r="G34" s="72"/>
+      <c r="H34" s="72"/>
+      <c r="I34" s="73"/>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="44" t="s">
+      <c r="B35" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="46"/>
+      <c r="C35" s="72"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="72"/>
+      <c r="F35" s="72"/>
+      <c r="G35" s="72"/>
+      <c r="H35" s="72"/>
+      <c r="I35" s="73"/>
     </row>
     <row r="36" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="44"/>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="45"/>
-      <c r="H36" s="45"/>
-      <c r="I36" s="46"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="72"/>
+      <c r="F36" s="72"/>
+      <c r="G36" s="72"/>
+      <c r="H36" s="72"/>
+      <c r="I36" s="73"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="44" t="s">
+      <c r="B37" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="45"/>
-      <c r="I37" s="46"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="72"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="73"/>
     </row>
     <row r="38" spans="2:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="44"/>
-      <c r="C38" s="45"/>
-      <c r="D38" s="45"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="45"/>
-      <c r="G38" s="45"/>
-      <c r="H38" s="45"/>
-      <c r="I38" s="46"/>
+      <c r="B38" s="71"/>
+      <c r="C38" s="72"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="72"/>
+      <c r="F38" s="72"/>
+      <c r="G38" s="72"/>
+      <c r="H38" s="72"/>
+      <c r="I38" s="73"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="44" t="s">
+      <c r="B39" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="45"/>
-      <c r="D39" s="45"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="45"/>
-      <c r="I39" s="46"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="72"/>
+      <c r="E39" s="72"/>
+      <c r="F39" s="72"/>
+      <c r="G39" s="72"/>
+      <c r="H39" s="72"/>
+      <c r="I39" s="73"/>
     </row>
     <row r="40" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="44"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="46"/>
+      <c r="B40" s="71"/>
+      <c r="C40" s="72"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="72"/>
+      <c r="F40" s="72"/>
+      <c r="G40" s="72"/>
+      <c r="H40" s="72"/>
+      <c r="I40" s="73"/>
     </row>
     <row r="41" spans="2:9" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="44" t="s">
+      <c r="B41" s="71" t="s">
         <v>28</v>
       </c>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
-      <c r="E41" s="45"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="45"/>
-      <c r="I41" s="46"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="72"/>
+      <c r="E41" s="72"/>
+      <c r="F41" s="72"/>
+      <c r="G41" s="72"/>
+      <c r="H41" s="72"/>
+      <c r="I41" s="73"/>
     </row>
     <row r="42" spans="2:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="44" t="s">
+      <c r="B42" s="71" t="s">
         <v>29</v>
       </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="45"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="46"/>
+      <c r="C42" s="72"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="72"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="73"/>
     </row>
     <row r="43" spans="2:9" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="41" t="s">
+      <c r="B43" s="105" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="42"/>
-      <c r="D43" s="42"/>
-      <c r="E43" s="42"/>
-      <c r="F43" s="42"/>
-      <c r="G43" s="42"/>
-      <c r="H43" s="42"/>
-      <c r="I43" s="43"/>
+      <c r="C43" s="106"/>
+      <c r="D43" s="106"/>
+      <c r="E43" s="106"/>
+      <c r="F43" s="106"/>
+      <c r="G43" s="106"/>
+      <c r="H43" s="106"/>
+      <c r="I43" s="107"/>
     </row>
     <row r="44" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="78" t="s">
+      <c r="B44" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="79"/>
-      <c r="D44" s="79"/>
-      <c r="E44" s="79"/>
-      <c r="F44" s="79"/>
-      <c r="G44" s="79"/>
-      <c r="H44" s="79"/>
-      <c r="I44" s="80"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="60"/>
+      <c r="E44" s="60"/>
+      <c r="F44" s="60"/>
+      <c r="G44" s="60"/>
+      <c r="H44" s="60"/>
+      <c r="I44" s="61"/>
     </row>
     <row r="45" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="54"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="55"/>
-      <c r="E45" s="55"/>
-      <c r="F45" s="55"/>
-      <c r="G45" s="55"/>
-      <c r="H45" s="55"/>
-      <c r="I45" s="56"/>
+      <c r="B45" s="79"/>
+      <c r="C45" s="80"/>
+      <c r="D45" s="80"/>
+      <c r="E45" s="80"/>
+      <c r="F45" s="80"/>
+      <c r="G45" s="80"/>
+      <c r="H45" s="80"/>
+      <c r="I45" s="81"/>
     </row>
     <row r="46" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="57"/>
-      <c r="C46" s="58"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="58"/>
-      <c r="G46" s="58"/>
-      <c r="H46" s="58"/>
-      <c r="I46" s="59"/>
+      <c r="B46" s="82"/>
+      <c r="C46" s="83"/>
+      <c r="D46" s="83"/>
+      <c r="E46" s="83"/>
+      <c r="F46" s="83"/>
+      <c r="G46" s="83"/>
+      <c r="H46" s="83"/>
+      <c r="I46" s="84"/>
     </row>
     <row r="47" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="57"/>
-      <c r="C47" s="58"/>
-      <c r="D47" s="58"/>
-      <c r="E47" s="58"/>
-      <c r="F47" s="58"/>
-      <c r="G47" s="58"/>
-      <c r="H47" s="58"/>
-      <c r="I47" s="59"/>
+      <c r="B47" s="82"/>
+      <c r="C47" s="83"/>
+      <c r="D47" s="83"/>
+      <c r="E47" s="83"/>
+      <c r="F47" s="83"/>
+      <c r="G47" s="83"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="84"/>
     </row>
     <row r="48" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="57"/>
-      <c r="C48" s="58"/>
-      <c r="D48" s="58"/>
-      <c r="E48" s="58"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="58"/>
-      <c r="H48" s="58"/>
-      <c r="I48" s="59"/>
+      <c r="B48" s="82"/>
+      <c r="C48" s="83"/>
+      <c r="D48" s="83"/>
+      <c r="E48" s="83"/>
+      <c r="F48" s="83"/>
+      <c r="G48" s="83"/>
+      <c r="H48" s="83"/>
+      <c r="I48" s="84"/>
     </row>
     <row r="49" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="57"/>
-      <c r="C49" s="58"/>
-      <c r="D49" s="58"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="58"/>
-      <c r="G49" s="58"/>
-      <c r="H49" s="58"/>
-      <c r="I49" s="59"/>
+      <c r="B49" s="82"/>
+      <c r="C49" s="83"/>
+      <c r="D49" s="83"/>
+      <c r="E49" s="83"/>
+      <c r="F49" s="83"/>
+      <c r="G49" s="83"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="84"/>
     </row>
     <row r="50" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="57"/>
-      <c r="C50" s="58"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="58"/>
-      <c r="H50" s="58"/>
-      <c r="I50" s="59"/>
+      <c r="B50" s="82"/>
+      <c r="C50" s="83"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="84"/>
     </row>
     <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="57"/>
-      <c r="C51" s="58"/>
-      <c r="D51" s="58"/>
-      <c r="E51" s="58"/>
-      <c r="F51" s="58"/>
-      <c r="G51" s="58"/>
-      <c r="H51" s="58"/>
-      <c r="I51" s="59"/>
+      <c r="B51" s="82"/>
+      <c r="C51" s="83"/>
+      <c r="D51" s="83"/>
+      <c r="E51" s="83"/>
+      <c r="F51" s="83"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="84"/>
     </row>
     <row r="52" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="60"/>
-      <c r="C52" s="61"/>
-      <c r="D52" s="61"/>
-      <c r="E52" s="61"/>
-      <c r="F52" s="61"/>
-      <c r="G52" s="61"/>
-      <c r="H52" s="61"/>
-      <c r="I52" s="62"/>
+      <c r="B52" s="85"/>
+      <c r="C52" s="86"/>
+      <c r="D52" s="86"/>
+      <c r="E52" s="86"/>
+      <c r="F52" s="86"/>
+      <c r="G52" s="86"/>
+      <c r="H52" s="86"/>
+      <c r="I52" s="87"/>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B53" s="63" t="s">
+      <c r="B53" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="C53" s="64"/>
-      <c r="D53" s="64"/>
-      <c r="E53" s="64"/>
-      <c r="F53" s="64"/>
-      <c r="G53" s="64"/>
-      <c r="H53" s="64"/>
-      <c r="I53" s="65"/>
+      <c r="C53" s="89"/>
+      <c r="D53" s="89"/>
+      <c r="E53" s="89"/>
+      <c r="F53" s="89"/>
+      <c r="G53" s="89"/>
+      <c r="H53" s="89"/>
+      <c r="I53" s="90"/>
     </row>
     <row r="54" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="66" t="s">
+      <c r="B54" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="C54" s="67"/>
-      <c r="D54" s="68" t="s">
+      <c r="C54" s="92"/>
+      <c r="D54" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="E54" s="68"/>
-      <c r="F54" s="68"/>
-      <c r="G54" s="69" t="s">
+      <c r="E54" s="93"/>
+      <c r="F54" s="93"/>
+      <c r="G54" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="H54" s="71"/>
-      <c r="I54" s="72"/>
+      <c r="H54" s="96"/>
+      <c r="I54" s="36"/>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B55" s="66" t="s">
+      <c r="B55" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C55" s="67"/>
-      <c r="D55" s="68" t="s">
+      <c r="C55" s="92"/>
+      <c r="D55" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="E55" s="68"/>
-      <c r="F55" s="68"/>
-      <c r="G55" s="69"/>
-      <c r="H55" s="71"/>
-      <c r="I55" s="72"/>
+      <c r="E55" s="93"/>
+      <c r="F55" s="93"/>
+      <c r="G55" s="94"/>
+      <c r="H55" s="96"/>
+      <c r="I55" s="36"/>
     </row>
     <row r="56" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="66"/>
-      <c r="C56" s="67"/>
-      <c r="D56" s="68"/>
-      <c r="E56" s="68"/>
-      <c r="F56" s="68"/>
-      <c r="G56" s="69"/>
-      <c r="H56" s="71"/>
-      <c r="I56" s="72"/>
+      <c r="B56" s="91"/>
+      <c r="C56" s="92"/>
+      <c r="D56" s="93"/>
+      <c r="E56" s="93"/>
+      <c r="F56" s="93"/>
+      <c r="G56" s="94"/>
+      <c r="H56" s="96"/>
+      <c r="I56" s="36"/>
     </row>
     <row r="57" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="63" t="s">
+      <c r="B57" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="C57" s="64"/>
-      <c r="D57" s="64"/>
-      <c r="E57" s="64"/>
-      <c r="F57" s="64"/>
-      <c r="G57" s="64"/>
-      <c r="H57" s="64"/>
-      <c r="I57" s="65"/>
+      <c r="C57" s="89"/>
+      <c r="D57" s="89"/>
+      <c r="E57" s="89"/>
+      <c r="F57" s="89"/>
+      <c r="G57" s="89"/>
+      <c r="H57" s="89"/>
+      <c r="I57" s="90"/>
     </row>
     <row r="58" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="66" t="s">
+      <c r="B58" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="C58" s="67"/>
-      <c r="D58" s="68">
+      <c r="C58" s="92"/>
+      <c r="D58" s="93">
         <f>E10</f>
         <v>0</v>
       </c>
-      <c r="E58" s="68"/>
-      <c r="F58" s="68"/>
-      <c r="G58" s="69" t="s">
+      <c r="E58" s="93"/>
+      <c r="F58" s="93"/>
+      <c r="G58" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="H58" s="71"/>
-      <c r="I58" s="72"/>
+      <c r="H58" s="96"/>
+      <c r="I58" s="36"/>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B59" s="66" t="s">
+      <c r="B59" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C59" s="67"/>
-      <c r="D59" s="68">
+      <c r="C59" s="92"/>
+      <c r="D59" s="93">
         <f>I10</f>
         <v>0</v>
       </c>
-      <c r="E59" s="68"/>
-      <c r="F59" s="68"/>
-      <c r="G59" s="69"/>
-      <c r="H59" s="71"/>
-      <c r="I59" s="72"/>
+      <c r="E59" s="93"/>
+      <c r="F59" s="93"/>
+      <c r="G59" s="94"/>
+      <c r="H59" s="96"/>
+      <c r="I59" s="36"/>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B60" s="75"/>
-      <c r="C60" s="76"/>
-      <c r="D60" s="77"/>
-      <c r="E60" s="77"/>
-      <c r="F60" s="77"/>
-      <c r="G60" s="70"/>
-      <c r="H60" s="73"/>
-      <c r="I60" s="74"/>
+      <c r="B60" s="98"/>
+      <c r="C60" s="99"/>
+      <c r="D60" s="100"/>
+      <c r="E60" s="100"/>
+      <c r="F60" s="100"/>
+      <c r="G60" s="95"/>
+      <c r="H60" s="97"/>
+      <c r="I60" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="75">
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="B1:C5"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="D2:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B31:I32"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B35:I36"/>
+    <mergeCell ref="B37:I38"/>
+    <mergeCell ref="B39:I40"/>
+    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B45:I52"/>
+    <mergeCell ref="B57:I57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="G58:G60"/>
+    <mergeCell ref="H58:I60"/>
+    <mergeCell ref="B59:C60"/>
+    <mergeCell ref="D59:F60"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="B55:C56"/>
+    <mergeCell ref="D55:F56"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="H54:I56"/>
+    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B44:I44"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B30:I30"/>
@@ -2673,64 +2698,37 @@
     <mergeCell ref="E6:I6"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B45:I52"/>
-    <mergeCell ref="B57:I57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="G58:G60"/>
-    <mergeCell ref="H58:I60"/>
-    <mergeCell ref="B59:C60"/>
-    <mergeCell ref="D59:F60"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="B55:C56"/>
-    <mergeCell ref="D55:F56"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="H54:I56"/>
-    <mergeCell ref="B53:I53"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B31:I32"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B35:I36"/>
-    <mergeCell ref="B37:I38"/>
-    <mergeCell ref="B39:I40"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B1:C5"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="D2:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.78740157480314965" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.62992125984251968" right="0.62992125984251968" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="47" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2983,21 +2981,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
-    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3022,9 +3019,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
+    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>